<commit_message>
data(swarm-disaster): G09-P3-B5 author complete workbooks
</commit_message>
<xml_diff>
--- a/config/swarm-disaster-generated/templates/SwarmDisaster.xlsx
+++ b/config/swarm-disaster-generated/templates/SwarmDisaster.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2553" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2550" uniqueCount="237">
   <si>
     <t>@table</t>
   </si>
@@ -197,7 +197,7 @@
     <t>SwarmDisasterArea</t>
   </si>
   <si>
-    <t>506e6b1ed8143838</t>
+    <t>a20f0adc29115821</t>
   </si>
   <si>
     <t>area_kind</t>
@@ -272,6 +272,9 @@
     <t>range=1..3</t>
   </si>
   <si>
+    <t>parser=split;separator=|;length=1..128</t>
+  </si>
+  <si>
     <t>SwarmDisasterChessboard</t>
   </si>
   <si>
@@ -332,9 +335,6 @@
     <t>range=-100..100</t>
   </si>
   <si>
-    <t>parser=split;separator=|;length=1..128</t>
-  </si>
-  <si>
     <t>SwarmDisasterMapNode</t>
   </si>
   <si>
@@ -521,7 +521,7 @@
     <t>SwarmDisasterCountdownDisarray</t>
   </si>
   <si>
-    <t>7013054f5eb4f81b</t>
+    <t>6aafe41b24ce8b30</t>
   </si>
   <si>
     <t>initial_value</t>
@@ -542,7 +542,7 @@
     <t>transition_boundary</t>
   </si>
   <si>
-    <t>transition_result</t>
+    <t>transition_result_json</t>
   </si>
   <si>
     <t>warning_threshold</t>
@@ -602,7 +602,7 @@
     <t>SwarmDisasterAudiencePath</t>
   </si>
   <si>
-    <t>8f459c52b32d3209</t>
+    <t>514e3b06169b703c</t>
   </si>
   <si>
     <t>sort</t>
@@ -644,7 +644,7 @@
     <t>SwarmDisasterAudienceDie</t>
   </si>
   <si>
-    <t>b0cc2adcc81ab2a5</t>
+    <t>0041beac2e670950</t>
   </si>
   <si>
     <t>audience_path_id</t>
@@ -1716,7 +1716,7 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>123</v>
@@ -1781,7 +1781,7 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>123</v>
@@ -1846,7 +1846,7 @@
         <v>36</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>36</v>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="R6" s="5"/>
       <c r="S6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="T6" s="5" t="s">
         <v>67</v>
@@ -3920,7 +3920,7 @@
         <v>46</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="42" customHeight="1">
@@ -3990,7 +3990,8 @@
     <col min="18" max="18" width="22.7109375" style="5" customWidth="1"/>
     <col min="19" max="19" width="12.7109375" style="5" customWidth="1"/>
     <col min="20" max="20" width="19.7109375" style="5" customWidth="1"/>
-    <col min="21" max="22" width="17.7109375" style="5" customWidth="1"/>
+    <col min="21" max="21" width="22.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="17.7109375" style="5" customWidth="1"/>
     <col min="23" max="23" width="19.7109375" style="5" customWidth="1"/>
     <col min="24" max="24" width="12.7109375" style="5" customWidth="1"/>
     <col min="25" max="25" width="19.7109375" style="5" customWidth="1"/>
@@ -4405,7 +4406,7 @@
         <v>114</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>114</v>
+        <v>67</v>
       </c>
       <c r="V6" s="5" t="s">
         <v>120</v>
@@ -4954,7 +4955,7 @@
     <col min="13" max="14" width="22.7109375" style="5" customWidth="1"/>
     <col min="15" max="17" width="12.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="32.7109375" style="5" customWidth="1"/>
-    <col min="19" max="19" width="12.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" style="5" customWidth="1"/>
     <col min="20" max="20" width="18.7109375" style="5" customWidth="1"/>
     <col min="21" max="22" width="20.7109375" style="5" customWidth="1"/>
     <col min="23" max="23" width="22.7109375" style="5" customWidth="1"/>
@@ -5218,7 +5219,7 @@
         <v>200</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="T4" s="5" t="s">
         <v>36</v>
@@ -5369,15 +5370,13 @@
         <v>63</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>46</v>
       </c>
       <c r="R6" s="5"/>
-      <c r="S6" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="S6" s="5"/>
       <c r="T6" s="5" t="s">
         <v>67</v>
       </c>
@@ -5474,8 +5473,7 @@
     <col min="15" max="16" width="12.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="32.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="12.7109375" style="5" customWidth="1"/>
-    <col min="19" max="19" width="16.7109375" style="5" customWidth="1"/>
-    <col min="20" max="20" width="12.7109375" style="5" customWidth="1"/>
+    <col min="19" max="20" width="16.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="25.7109375" style="5" customWidth="1"/>
     <col min="22" max="22" width="28.7109375" style="5" customWidth="1"/>
     <col min="23" max="23" width="25.7109375" style="5" customWidth="1"/>
@@ -5728,7 +5726,7 @@
         <v>36</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>36</v>
@@ -5873,9 +5871,7 @@
       <c r="S6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="T6" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="T6" s="5"/>
       <c r="U6" s="5" t="s">
         <v>186</v>
       </c>
@@ -5956,7 +5952,8 @@
     <col min="13" max="14" width="22.7109375" style="5" customWidth="1"/>
     <col min="15" max="17" width="12.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="22.7109375" style="5" customWidth="1"/>
-    <col min="19" max="20" width="12.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="12.7109375" style="5" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="17.7109375" style="5" customWidth="1"/>
     <col min="22" max="22" width="20.7109375" style="5" customWidth="1"/>
     <col min="23" max="23" width="23.7109375" style="5" customWidth="1"/>
@@ -6202,7 +6199,7 @@
         <v>62</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="U4" s="5" t="s">
         <v>35</v>
@@ -6343,9 +6340,7 @@
       <c r="S6" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="T6" s="5" t="s">
-        <v>63</v>
-      </c>
+      <c r="T6" s="5"/>
       <c r="U6" s="5" t="s">
         <v>66</v>
       </c>
@@ -6767,11 +6762,11 @@
       </c>
       <c r="P6" s="5"/>
       <c r="Q6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="R6" s="5"/>
       <c r="S6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="T6" s="5"/>
       <c r="U6" s="5" t="s">
@@ -8632,7 +8627,7 @@
         <v>77</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>64</v>
+        <v>78</v>
       </c>
       <c r="R6" s="5" t="s">
         <v>47</v>
@@ -8709,7 +8704,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -8733,7 +8728,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="24" customHeight="1">
@@ -8783,25 +8778,25 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:22">
@@ -8851,25 +8846,25 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:22">
@@ -8925,10 +8920,10 @@
         <v>35</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="T4" s="5" t="s">
         <v>36</v>
@@ -9049,10 +9044,10 @@
         <v>63</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
@@ -9142,7 +9137,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -9166,7 +9161,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -9213,16 +9208,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -9269,16 +9264,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -9325,7 +9320,7 @@
         <v>40</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P4" s="5" t="s">
         <v>35</v>
@@ -9432,13 +9427,13 @@
       </c>
       <c r="O6" s="5"/>
       <c r="P6" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
@@ -9592,13 +9587,13 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>101</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S2" s="3" t="s">
         <v>102</v>
@@ -9663,13 +9658,13 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>101</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>102</v>
@@ -9734,7 +9729,7 @@
         <v>36</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>107</v>
@@ -9872,10 +9867,10 @@
       <c r="P6" s="5"/>
       <c r="Q6" s="5"/>
       <c r="R6" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="T6" s="5" t="s">
         <v>50</v>
@@ -10041,7 +10036,7 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P2" s="3" t="s">
         <v>111</v>
@@ -10097,7 +10092,7 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="P3" s="5" t="s">
         <v>111</v>
@@ -10153,13 +10148,13 @@
         <v>40</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>36</v>
@@ -10405,7 +10400,7 @@
         <v>24</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>117</v>
@@ -10464,7 +10459,7 @@
         <v>24</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>117</v>
@@ -10523,7 +10518,7 @@
         <v>36</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>36</v>

</xml_diff>